<commit_message>
Report UI, PDF, Excel exports for 4 scales
</commit_message>
<xml_diff>
--- a/forms/app/ddst.xlsx
+++ b/forms/app/ddst.xlsx
@@ -4305,7 +4305,7 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>86. Understand 4 Prepositions</t>
+          <t>86. Understand 4 Prepositions [AGE UNCONFIRMED — TODO]</t>
         </is>
       </c>
       <c r="D120" t="inlineStr"/>
@@ -4317,7 +4317,7 @@
       <c r="F120" t="inlineStr"/>
       <c r="G120" t="inlineStr">
         <is>
-          <t>${show_all} = 'yes' or ${ca_months_dec} &gt;= 56.0000</t>
+          <t>true()</t>
         </is>
       </c>
       <c r="H120" t="inlineStr"/>
@@ -4339,7 +4339,7 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>87. Speech Fully Understandable</t>
+          <t>87. Speech Fully Understandable [AGE UNCONFIRMED — TODO]</t>
         </is>
       </c>
       <c r="D121" t="inlineStr"/>
@@ -4351,7 +4351,7 @@
       <c r="F121" t="inlineStr"/>
       <c r="G121" t="inlineStr">
         <is>
-          <t>${show_all} = 'yes' or ${ca_months_dec} &gt;= 51.0000</t>
+          <t>true()</t>
         </is>
       </c>
       <c r="H121" t="inlineStr"/>
@@ -4373,7 +4373,7 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>88. Define 3 Words</t>
+          <t>88. Define 3 Words [AGE UNCONFIRMED — TODO]</t>
         </is>
       </c>
       <c r="D122" t="inlineStr"/>
@@ -4385,7 +4385,7 @@
       <c r="F122" t="inlineStr"/>
       <c r="G122" t="inlineStr">
         <is>
-          <t>${show_all} = 'yes' or ${ca_months_dec} &gt;= 64.0000</t>
+          <t>true()</t>
         </is>
       </c>
       <c r="H122" t="inlineStr"/>
@@ -4543,7 +4543,7 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>93. Name 4 Colors</t>
+          <t>93. Language Item 39 — row count reconciliation [AGE UNCONFIRMED] [AGE UNCONFIRMED — TODO]</t>
         </is>
       </c>
       <c r="D127" t="inlineStr"/>
@@ -4555,7 +4555,7 @@
       <c r="F127" t="inlineStr"/>
       <c r="G127" t="inlineStr">
         <is>
-          <t>${show_all} = 'yes' or ${ca_months_dec} &gt;= 62.0000</t>
+          <t>true()</t>
         </is>
       </c>
       <c r="H127" t="inlineStr"/>
@@ -7982,7 +7982,7 @@
       <c r="I249" t="inlineStr"/>
       <c r="J249" t="inlineStr">
         <is>
-          <t>if((selected(${lang_32}, 'F') or selected(${lang_32}, 'R')) and ${ca_months_dec} &gt;= 56.0, 1, 0)</t>
+          <t>0</t>
         </is>
       </c>
       <c r="K249" t="inlineStr"/>
@@ -8008,7 +8008,7 @@
       <c r="I250" t="inlineStr"/>
       <c r="J250" t="inlineStr">
         <is>
-          <t>if((selected(${lang_33}, 'F') or selected(${lang_33}, 'R')) and ${ca_months_dec} &gt;= 51.0, 1, 0)</t>
+          <t>0</t>
         </is>
       </c>
       <c r="K250" t="inlineStr"/>
@@ -8034,7 +8034,7 @@
       <c r="I251" t="inlineStr"/>
       <c r="J251" t="inlineStr">
         <is>
-          <t>if((selected(${lang_34}, 'F') or selected(${lang_34}, 'R')) and ${ca_months_dec} &gt;= 64.0, 1, 0)</t>
+          <t>0</t>
         </is>
       </c>
       <c r="K251" t="inlineStr"/>
@@ -8164,7 +8164,7 @@
       <c r="I256" t="inlineStr"/>
       <c r="J256" t="inlineStr">
         <is>
-          <t>if((selected(${lang_39}, 'F') or selected(${lang_39}, 'R')) and ${ca_months_dec} &gt;= 62.0, 1, 0)</t>
+          <t>0</t>
         </is>
       </c>
       <c r="K256" t="inlineStr"/>

</xml_diff>